<commit_message>
update(TechBytes): consolidated website directory (21 unique websites) - 2026-10-25 10:09:19
</commit_message>
<xml_diff>
--- a/📁 TechBytes/📊 TechBytes_Websites_Master_List.xlsx
+++ b/📁 TechBytes/📊 TechBytes_Websites_Master_List.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -521,25 +521,25 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Before you drop $600 on headphones</t>
+          <t>MuscleWiki</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>https://tinywow.com</t>
+          <t>https://musclewiki.com</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Online productivity utilities: Before you drop $600 on headphones • Online productivity utilities: Is this the worlds smallest PC? • Online productivity utilities: Keychron Q3 Ultra 8K keyboard unboxing • Online productivity utilities: Honor 600 Pro unboxing (Channel me kul 349 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Interactive visual body map where you click any muscle to get exercise guides and workout plans. (Channel me kul 3 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>349</v>
+        <v>3</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>349 videos (Primary: https://www.youtube.com/shorts/N-6ADl4gkYk)</t>
+          <t>3 videos (Primary: https://www.youtube.com/shorts/PKCFZ3WJrug)</t>
         </is>
       </c>
     </row>
@@ -551,25 +551,25 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>MuscleWiki</t>
+          <t>SuperCook</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://musclewiki.com</t>
+          <t>https://supercook.com</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive visual body map where you click any muscle to get exercise guides and workout plans. (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Zero-waste recipe search engine that matches recipes to ingredients you already have at home.</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/PKCFZ3WJrug)</t>
+          <t>More variety, less food wastage!! Win win (https://www.youtube.com/shorts/q9QA9_ichTE)</t>
         </is>
       </c>
     </row>
@@ -581,25 +581,25 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SuperCook</t>
+          <t>TinyWow</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>https://supercook.com</t>
+          <t>https://tinywow.com</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Zero-waste recipe search engine that matches recipes to ingredients you already have at home.</t>
+          <t>Is website se ye sab kar sakte hain: 200+ free online utility tools: PDF editing/converting/merging, image background removal, file compression, video tools, and AI writing. (Channel me kul 317 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1</v>
+        <v>317</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>More variety, less food wastage!! Win win (https://www.youtube.com/shorts/q9QA9_ichTE)</t>
+          <t>317 videos (Primary: https://www.youtube.com/shorts/N-6ADl4gkYk)</t>
         </is>
       </c>
     </row>
@@ -641,25 +641,25 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Find and buy car parts for any</t>
+          <t>Looka AI</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://toools.design</t>
+          <t>https://looka.com</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Creative design utility: Find and buy car parts for any vehicle in seconds! • Creative design utility: Edit photos in seconds! • Creative design utility: Find car parts to repair your car! • Creative design utility: Transform your photo to video in seconds! (Channel me kul 261 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: AI-powered logo designer and brand identity generator with complete marketing packages.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>261</v>
+        <v>1</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>261 videos (Primary: https://www.youtube.com/shorts/fkBn34HO7a0)</t>
+          <t>AI generates logos in seconds! RIP logo designers (https://www.youtube.com/shorts/UzP8KhBI5qE)</t>
         </is>
       </c>
     </row>
@@ -671,25 +671,25 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Looka AI</t>
+          <t>MockupBro</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>https://looka.com</t>
+          <t>https://mockupbro.com</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI-powered logo designer and brand identity generator with complete marketing packages.</t>
+          <t>Is website se ye kar sakte hain: Free online device and product mockup generator with high-resolution instant downloads. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>AI generates logos in seconds! RIP logo designers (https://www.youtube.com/shorts/UzP8KhBI5qE)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/tiHtqPN3ui4)</t>
         </is>
       </c>
     </row>
@@ -701,25 +701,25 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MockupBro</t>
+          <t>Papercurves</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>https://mockupbro.com</t>
+          <t>https://papercurves.com</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Free online device and product mockup generator with high-resolution instant downloads. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Interactive 3D paper fold and flip animation generator for creative web interfaces.</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/tiHtqPN3ui4)</t>
+          <t>Create paper animations in seconds! (https://www.youtube.com/shorts/RwHjRKG2opI)</t>
         </is>
       </c>
     </row>
@@ -731,25 +731,25 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Papercurves</t>
+          <t>Remove.bg</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>https://papercurves.com</t>
+          <t>https://remove.bg</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive 3D paper fold and flip animation generator for creative web interfaces.</t>
+          <t>Is website se ye sab kar sakte hain: 1-click automated AI tool to remove image backgrounds with high-precision edge cutout in seconds. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Create paper animations in seconds! (https://www.youtube.com/shorts/RwHjRKG2opI)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/LAyS5YejzKk)</t>
         </is>
       </c>
     </row>
@@ -761,25 +761,25 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Remove.bg</t>
+          <t>Toools.design</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>https://remove.bg</t>
+          <t>https://toools.design</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: 1-click automated AI tool to remove image backgrounds with high-precision edge cutout. (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Curated repository of 1,000+ modern design tools, mockups, typography, illustration packs, and UI kits. (Channel me kul 283 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2</v>
+        <v>283</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/LAyS5YejzKk)</t>
+          <t>283 videos (Primary: https://www.youtube.com/shorts/NseLXXWmPMs)</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Turn a song into a cinematic m</t>
+          <t>Vocal Remover</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -801,15 +801,15 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Audio manipulation: Turn a song into a cinematic music video in seconds! • Audio manipulation: Create a song in seconds! • Audio manipulation: Create songs and music in seconds! • Audio manipulation: Play song trivia with your friends! (Channel me kul 5 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: AI-powered online audio tool that isolates vocals and instrumental tracks for free. (Channel me kul 10 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>5 videos (Primary: https://www.youtube.com/shorts/SLhccBVbIHs)</t>
+          <t>10 videos (Primary: https://www.youtube.com/shorts/SLhccBVbIHs)</t>
         </is>
       </c>
     </row>
@@ -821,25 +821,25 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Apple watch ultra 3 unboxing w</t>
+          <t>Framer</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>https://replit.com</t>
+          <t>https://framer.com</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Development &amp; code features: Apple Watch Ultra 3 unboxing with the Milanese strap • Development &amp; code features: Build a working app in seconds! • Development &amp; code features: Create web and apps designs in seconds! • Development &amp; code features: Learning to code WAS boring this website makes learning coding interactive and fun! (Channel me kul 11 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: AI-powered no-code website builder that creates responsive production-ready sites.</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>11 videos (Primary: https://www.youtube.com/shorts/Xv2yl3HgOnk)</t>
+          <t>Design and build a website in minutes! (https://www.youtube.com/shorts/H2yimEjbagg)</t>
         </is>
       </c>
     </row>
@@ -851,25 +851,25 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Framer</t>
+          <t>Replit</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://framer.com</t>
+          <t>https://replit.com</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: AI-powered no-code website builder that creates responsive production-ready sites.</t>
+          <t>Is website se ye sab kar sakte hain: Collaborative browser-based IDE, AI code generation, and instant cloud application deployment workspace. (Channel me kul 10 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Design and build a website in minutes! (https://www.youtube.com/shorts/H2yimEjbagg)</t>
+          <t>10 videos (Primary: https://www.youtube.com/shorts/Xv2yl3HgOnk)</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Interactive 3D model of the human anatomy, diseases, and medical treatments.</t>
+          <t>Is website se ye sab kar sakte hain: Interactive 3D virtual human anatomy atlas and disease explorer for medical students, healthcare pros, and biology.</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -911,55 +911,55 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Wallpapers you need dragon bal</t>
+          <t>Coursera</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>https://quillbot.com</t>
+          <t>https://coursera.org</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Study &amp; academic utility: Wallpapers you need dragon ball z edition • Study &amp; academic utility: This interactive wallpaper is dope! • Study &amp; academic utility: Wallpapers you need, black and white edition • Study &amp; academic utility: Create AI wallpapers in seconds (Channel me kul 10 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: Global online learning platform offering courses and degrees from top universities like Stanford and Yale.</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>10 videos (Primary: https://www.youtube.com/shorts/X4GWMnywb5U)</t>
+          <t>Find roadmaps for your next programming career! (https://www.youtube.com/shorts/JYyE4AlfQXg)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>🗺️ Maps, 3D &amp; Exploration</t>
+          <t>📚 Learning, Study &amp; Research</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Flightradar24</t>
+          <t>QuillBot</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>https://flightradar24.com</t>
+          <t>https://quillbot.com</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Real-time global aircraft and flight tracker with detailed flight route data.</t>
+          <t>Is website se ye sab kar sakte hain: AI paraphrasing, grammar checking, academic summarization, plagiarism detection, and student thesis writing assistance. (Channel me kul 10 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>See live flight details from around the world! (https://www.youtube.com/shorts/GAJzEF8IwXo)</t>
+          <t>10 videos (Primary: https://www.youtube.com/shorts/X4GWMnywb5U)</t>
         </is>
       </c>
     </row>
@@ -971,25 +971,25 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>The True Size Of</t>
+          <t>EarthCam</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>https://thetruesize.com</t>
+          <t>https://earthcam.com</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Drag countries across the globe to discover their true scale without map distortion.</t>
+          <t>Is website se ye sab kar sakte hain: Global network of live streaming webcams providing scenic and landmark views worldwide. (Channel me kul 8 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Compare the true size of each country! (https://www.youtube.com/shorts/2iRkaOAqQoI)</t>
+          <t>8 videos (Primary: https://www.youtube.com/shorts/aKkIdMQEiAs)</t>
         </is>
       </c>
     </row>
@@ -1001,55 +1001,55 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Travel planning in seconds!</t>
+          <t>Flightradar24</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>https://earthcam.com</t>
+          <t>https://flightradar24.com</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Interactive map &amp; location views: Travel planning in seconds! • Interactive map &amp; location views: Animate your next travel plan • Interactive map &amp; location views: Charge your tech on the go! Plenty of storage! Ready for travel thanks to (Channel me kul 3 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Real-time global aircraft and flight tracker with detailed flight route data.</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>3 videos (Primary: https://www.youtube.com/shorts/UPoUfOMpTtc)</t>
+          <t>See live flight details from around the world! (https://www.youtube.com/shorts/GAJzEF8IwXo)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>🤖 AI &amp; Machine Learning Tools</t>
+          <t>🗺️ Maps, 3D &amp; Exploration</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Predis.ai</t>
+          <t>The True Size Of</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>https://predis.ai</t>
+          <t>https://thetruesize.com</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Online web application: Predis.ai (Channel me kul 2 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: Drag countries across the globe to discover their true scale without map distortion.</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>2 videos (Primary: https://www.youtube.com/shorts/0pwRucBrg9Y)</t>
+          <t>Compare the true size of each country! (https://www.youtube.com/shorts/2iRkaOAqQoI)</t>
         </is>
       </c>
     </row>
@@ -1061,25 +1061,85 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>This bottle is self cleaning!</t>
+          <t>ChatGPT</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
+          <t>https://chatgpt.com</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Conversational AI assistant by OpenAI for answering questions, coding, research, writing, and problem solving. (Channel me kul 7 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>7 videos (Primary: https://www.youtube.com/shorts/DpvkjUEtruM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Predis.ai</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>https://predis.ai</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Is website se ye kar sakte hain: Online web application: Predis.ai</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Marketers will love Predis.ai! Analyse your competitors social posts for free. Link in bio (https://www.youtube.com/shorts/0pwRucBrg9Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Toolify.ai</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
           <t>https://toolify.ai</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Is website se ye sab kar sakte hain: AI features: This bottle is self cleaning! • AI features: Generate videos from a prompt in seconds! • AI features: This is like ChatGPT but stealth?! • AI features: This bottle purifies and filters your water (Channel me kul 19 alag-alag videos me featured)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>19 videos (Primary: https://www.youtube.com/shorts/IslF7Oh5Jio)</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Comprehensive global directory and discovery engine indexing 10,000+ AI software tools, models, and apps updated daily. (Channel me kul 13 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>13 videos (Primary: https://www.youtube.com/shorts/IslF7Oh5Jio)</t>
         </is>
       </c>
     </row>
@@ -1104,6 +1164,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>